<commit_message>
chore: seed workbook with blank computed fields
</commit_message>
<xml_diff>
--- a/sources/Public Invention Projects.xlsx
+++ b/sources/Public Invention Projects.xlsx
@@ -1852,9 +1852,7 @@
       <c r="A2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B2" s="8"/>
       <c r="C2" s="7" t="s">
         <v>13</v>
       </c>
@@ -1881,24 +1879,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M2"/>
+      <c r="N2"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B3" s="8"/>
       <c r="C3" s="7" t="s">
         <v>19</v>
       </c>
@@ -1925,24 +1913,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M3"/>
+      <c r="N3"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B4" s="8"/>
       <c r="C4" s="7" t="s">
         <v>23</v>
       </c>
@@ -1969,24 +1947,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M4"/>
+      <c r="N4"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B5" s="8"/>
       <c r="C5" s="7" t="s">
         <v>27</v>
       </c>
@@ -2013,24 +1981,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M5"/>
+      <c r="N5"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B6" s="8"/>
       <c r="C6" s="7" t="s">
         <v>31</v>
       </c>
@@ -2057,24 +2015,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M6"/>
+      <c r="N6"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B7" s="8"/>
       <c r="C7" s="7" t="s">
         <v>31</v>
       </c>
@@ -2101,24 +2049,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M7"/>
+      <c r="N7"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B8" s="8"/>
       <c r="C8" s="7" t="s">
         <v>38</v>
       </c>
@@ -2145,24 +2083,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M8"/>
+      <c r="N8"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B9" s="8"/>
       <c r="C9" s="7" t="s">
         <v>42</v>
       </c>
@@ -2189,24 +2117,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M9"/>
+      <c r="N9"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B10" s="8"/>
       <c r="C10" s="7" t="s">
         <v>46</v>
       </c>
@@ -2233,24 +2151,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M10"/>
+      <c r="N10"/>
     </row>
     <row r="11" ht="28.5" customHeight="1">
       <c r="A11" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="B11" s="8"/>
       <c r="C11" s="7" t="s">
         <v>51</v>
       </c>
@@ -2283,24 +2191,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-05-27T03:06:59Z</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M11"/>
+      <c r="N11"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B12" s="8"/>
       <c r="C12" s="7" t="s">
         <v>56</v>
       </c>
@@ -2333,24 +2231,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M12"/>
+      <c r="N12"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B13" s="8"/>
       <c r="C13" s="7" t="s">
         <v>60</v>
       </c>
@@ -2377,24 +2265,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M13"/>
+      <c r="N13"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B14" s="8"/>
       <c r="C14" s="7" t="s">
         <v>64</v>
       </c>
@@ -2421,24 +2299,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M14"/>
+      <c r="N14"/>
     </row>
     <row r="15" ht="29.25" customHeight="1">
       <c r="A15" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B15" s="8"/>
       <c r="C15" s="7" t="s">
         <v>68</v>
       </c>
@@ -2465,24 +2333,14 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2020-06-04T23:47:07Z</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M15"/>
+      <c r="N15"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="B16" s="8"/>
       <c r="C16" s="7" t="s">
         <v>73</v>
       </c>
@@ -2515,24 +2373,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M16"/>
+      <c r="N16"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B17" s="8"/>
       <c r="C17" s="7" t="s">
         <v>77</v>
       </c>
@@ -2559,24 +2407,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M17"/>
+      <c r="N17"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="B18" s="8"/>
       <c r="C18" s="7" t="s">
         <v>81</v>
       </c>
@@ -2609,24 +2447,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>2026-06-07T06:29:57Z</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M18"/>
+      <c r="N18"/>
     </row>
     <row r="19" ht="42.75" customHeight="1">
       <c r="A19" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="B19" s="8"/>
       <c r="C19" s="7" t="s">
         <v>85</v>
       </c>
@@ -2659,24 +2487,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2026-06-03T17:01:17Z</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M19"/>
+      <c r="N19"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B20" s="8"/>
       <c r="C20" s="7" t="s">
         <v>89</v>
       </c>
@@ -2703,24 +2521,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M20"/>
+      <c r="N20"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B21" s="8"/>
       <c r="C21" s="7" t="s">
         <v>94</v>
       </c>
@@ -2747,24 +2555,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M21"/>
+      <c r="N21"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B22" s="8"/>
       <c r="C22" s="7" t="s">
         <v>98</v>
       </c>
@@ -2791,24 +2589,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M22"/>
+      <c r="N22"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B23" s="8"/>
       <c r="C23" s="7" t="s">
         <v>102</v>
       </c>
@@ -2835,24 +2623,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M23"/>
+      <c r="N23"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B24" s="8"/>
       <c r="C24" s="7" t="s">
         <v>107</v>
       </c>
@@ -2879,24 +2657,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M24"/>
+      <c r="N24"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="B25" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B25" s="8"/>
       <c r="C25" s="7" t="s">
         <v>110</v>
       </c>
@@ -2923,24 +2691,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M25"/>
+      <c r="N25"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="B26" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B26" s="8"/>
       <c r="C26" s="7" t="s">
         <v>115</v>
       </c>
@@ -2967,24 +2725,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M26"/>
+      <c r="N26"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B27" s="8"/>
       <c r="C27" s="7" t="s">
         <v>120</v>
       </c>
@@ -3009,24 +2757,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M27"/>
+      <c r="N27"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="B28" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B28" s="8"/>
       <c r="C28" s="7" t="s">
         <v>123</v>
       </c>
@@ -3053,24 +2791,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M28"/>
+      <c r="N28"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B29" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B29" s="8"/>
       <c r="C29" s="7" t="s">
         <v>127</v>
       </c>
@@ -3097,24 +2825,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M29"/>
+      <c r="N29"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B30" s="15" t="s">
-        <v>50</v>
-      </c>
+      <c r="B30" s="15"/>
       <c r="C30" s="7" t="s">
         <v>131</v>
       </c>
@@ -3147,24 +2865,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>2026-05-13T20:17:27Z</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M30"/>
+      <c r="N30"/>
     </row>
     <row r="31" ht="41.25" customHeight="1">
       <c r="A31" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="B31" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B31" s="8"/>
       <c r="C31" s="7" t="s">
         <v>136</v>
       </c>
@@ -3191,24 +2899,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M31"/>
+      <c r="N31"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B32" s="8"/>
       <c r="C32" s="7" t="s">
         <v>140</v>
       </c>
@@ -3235,24 +2933,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M32"/>
+      <c r="N32"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="B33" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="B33" s="15"/>
       <c r="C33" s="7" t="s">
         <v>146</v>
       </c>
@@ -3279,24 +2967,14 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>2024-10-19T22:22:05Z</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M33"/>
+      <c r="N33"/>
     </row>
     <row r="34" ht="33.0" customHeight="1">
       <c r="A34" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B34" s="8"/>
       <c r="C34" s="7" t="s">
         <v>150</v>
       </c>
@@ -3323,24 +3001,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M34"/>
+      <c r="N34"/>
     </row>
     <row r="35" ht="29.25" customHeight="1">
       <c r="A35" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="B35" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B35" s="8"/>
       <c r="C35" s="7" t="s">
         <v>154</v>
       </c>
@@ -3368,19 +3036,13 @@
         </is>
       </c>
       <c r="M35"/>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>non_github</t>
-        </is>
-      </c>
+      <c r="N35"/>
     </row>
     <row r="37" ht="31.5" customHeight="1">
       <c r="A37" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="B37" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B37" s="8"/>
       <c r="C37" s="7" t="s">
         <v>159</v>
       </c>
@@ -3407,24 +3069,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M37"/>
+      <c r="N37"/>
     </row>
     <row r="38" ht="27.75" customHeight="1">
       <c r="A38" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="B38" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="B38" s="8"/>
       <c r="C38" s="7" t="s">
         <v>163</v>
       </c>
@@ -3457,24 +3109,14 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>2023-09-07T16:17:15Z</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M38"/>
+      <c r="N38"/>
     </row>
     <row r="39" ht="31.5" customHeight="1">
       <c r="A39" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="B39" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="B39" s="8"/>
       <c r="C39" s="7" t="s">
         <v>167</v>
       </c>
@@ -3507,24 +3149,14 @@
           <t>Stale</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>2025-09-04T19:12:30Z</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M39"/>
+      <c r="N39"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="B40" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="B40" s="15"/>
       <c r="C40" s="7" t="s">
         <v>171</v>
       </c>
@@ -3552,19 +3184,13 @@
         </is>
       </c>
       <c r="M40"/>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>non_github</t>
-        </is>
-      </c>
+      <c r="N40"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="B41" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B41" s="8"/>
       <c r="C41" s="7" t="s">
         <v>175</v>
       </c>
@@ -3590,19 +3216,13 @@
         </is>
       </c>
       <c r="M41"/>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+      <c r="N41"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="B42" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B42" s="8"/>
       <c r="C42" s="7" t="s">
         <v>178</v>
       </c>
@@ -3628,19 +3248,13 @@
         </is>
       </c>
       <c r="M42"/>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+      <c r="N42"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="B43" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B43" s="8"/>
       <c r="C43" s="7" t="s">
         <v>181</v>
       </c>
@@ -3666,19 +3280,13 @@
         </is>
       </c>
       <c r="M43"/>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+      <c r="N43"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="B44" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B44" s="8"/>
       <c r="C44" s="7" t="s">
         <v>184</v>
       </c>
@@ -3700,24 +3308,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M44"/>
+      <c r="N44"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="B45" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="B45" s="8"/>
       <c r="C45" s="7" t="s">
         <v>187</v>
       </c>
@@ -3750,24 +3348,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M45"/>
+      <c r="N45"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="B46" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="B46" s="15"/>
       <c r="C46" s="7" t="s">
         <v>191</v>
       </c>
@@ -3800,24 +3388,14 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>2021-08-25T21:55:35Z</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M46"/>
+      <c r="N46"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="B47" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B47" s="8"/>
       <c r="C47" s="7" t="s">
         <v>195</v>
       </c>
@@ -3844,24 +3422,14 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>2021-06-08T02:13:06Z</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M47"/>
+      <c r="N47"/>
     </row>
     <row r="48" ht="27.0" customHeight="1">
       <c r="A48" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="B48" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="B48" s="8"/>
       <c r="C48" s="7" t="s">
         <v>199</v>
       </c>
@@ -3888,24 +3456,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M48"/>
+      <c r="N48"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="B49" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B49" s="8"/>
       <c r="C49" s="7" t="s">
         <v>203</v>
       </c>
@@ -3932,24 +3490,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M49"/>
+      <c r="N49"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="B50" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B50" s="8"/>
       <c r="C50" s="7" t="s">
         <v>207</v>
       </c>
@@ -3976,24 +3524,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M50"/>
+      <c r="N50"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="B51" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="B51" s="15"/>
       <c r="C51" s="7" t="s">
         <v>211</v>
       </c>
@@ -4020,24 +3558,14 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>2023-01-06T21:26:13Z</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M51"/>
+      <c r="N51"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="B52" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="B52" s="15"/>
       <c r="C52" s="7" t="s">
         <v>216</v>
       </c>
@@ -4062,24 +3590,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>2026-05-13T20:17:27Z</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M52"/>
+      <c r="N52"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="B53" s="15" t="s">
-        <v>18</v>
-      </c>
+      <c r="B53" s="15"/>
       <c r="C53" s="7" t="s">
         <v>218</v>
       </c>
@@ -4104,24 +3622,14 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>2021-08-17T19:18:24Z</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M53"/>
+      <c r="N53"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="B54" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B54" s="8"/>
       <c r="C54" s="7" t="s">
         <v>221</v>
       </c>
@@ -4148,24 +3656,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M54"/>
+      <c r="N54"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="B55" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="B55" s="15"/>
       <c r="C55" s="7" t="s">
         <v>225</v>
       </c>
@@ -4199,19 +3697,13 @@
         </is>
       </c>
       <c r="M55"/>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>non_github</t>
-        </is>
-      </c>
+      <c r="N55"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="B56" s="15" t="s">
-        <v>50</v>
-      </c>
+      <c r="B56" s="15"/>
       <c r="C56" s="7" t="s">
         <v>230</v>
       </c>
@@ -4244,24 +3736,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>2026-06-05T20:13:32Z</t>
-        </is>
-      </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M56"/>
+      <c r="N56"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="B57" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B57" s="8"/>
       <c r="C57" s="7" t="s">
         <v>234</v>
       </c>
@@ -4287,19 +3769,13 @@
         </is>
       </c>
       <c r="M57"/>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+      <c r="N57"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="B58" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B58" s="8"/>
       <c r="C58" s="7" t="s">
         <v>237</v>
       </c>
@@ -4325,19 +3801,13 @@
         </is>
       </c>
       <c r="M58"/>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+      <c r="N58"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="B59" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="B59" s="15"/>
       <c r="C59" s="7" t="s">
         <v>240</v>
       </c>
@@ -4364,24 +3834,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>2026-05-04T02:42:30Z</t>
-        </is>
-      </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M59"/>
+      <c r="N59"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="8" t="s">
         <v>243</v>
       </c>
-      <c r="B60" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B60" s="8"/>
       <c r="C60" s="7" t="s">
         <v>244</v>
       </c>
@@ -4408,24 +3868,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M60"/>
+      <c r="N60"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="B61" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="B61" s="15"/>
       <c r="C61" s="7" t="s">
         <v>248</v>
       </c>
@@ -4452,24 +3902,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>2026-05-08T15:55:08Z</t>
-        </is>
-      </c>
-      <c r="N61" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M61"/>
+      <c r="N61"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="B62" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B62" s="8"/>
       <c r="C62" s="7" t="s">
         <v>252</v>
       </c>
@@ -4496,24 +3936,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M62"/>
+      <c r="N62"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="8" t="s">
         <v>255</v>
       </c>
-      <c r="B63" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B63" s="8"/>
       <c r="C63" s="7" t="s">
         <v>256</v>
       </c>
@@ -4540,24 +3970,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M63"/>
+      <c r="N63"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="B64" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="B64" s="15"/>
       <c r="C64" s="7" t="s">
         <v>260</v>
       </c>
@@ -4584,24 +4004,14 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>2023-06-16T02:35:10Z</t>
-        </is>
-      </c>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M64"/>
+      <c r="N64"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="15" t="s">
         <v>263</v>
       </c>
-      <c r="B65" s="15" t="s">
-        <v>50</v>
-      </c>
+      <c r="B65" s="15"/>
       <c r="C65" s="7" t="s">
         <v>264</v>
       </c>
@@ -4634,24 +4044,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t>2026-05-29T05:03:52Z</t>
-        </is>
-      </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M65"/>
+      <c r="N65"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="B66" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B66" s="8"/>
       <c r="C66" s="7" t="s">
         <v>268</v>
       </c>
@@ -4678,24 +4078,14 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>2024-05-18T01:55:34Z</t>
-        </is>
-      </c>
-      <c r="N66" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M66"/>
+      <c r="N66"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="B67" s="15" t="s">
-        <v>50</v>
-      </c>
+      <c r="B67" s="15"/>
       <c r="C67" s="19" t="s">
         <v>272</v>
       </c>
@@ -4728,24 +4118,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>2026-02-17T23:29:01Z</t>
-        </is>
-      </c>
-      <c r="N67" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="M67"/>
+      <c r="N67"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="21" t="s">
         <v>275</v>
       </c>
-      <c r="B68" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B68" s="8"/>
       <c r="C68" s="19" t="s">
         <v>276</v>
       </c>
@@ -4772,24 +4152,14 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M68"/>
+      <c r="N68"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="21" t="s">
         <v>279</v>
       </c>
-      <c r="B69" s="15" t="s">
-        <v>50</v>
-      </c>
+      <c r="B69" s="15"/>
       <c r="C69" s="19" t="s">
         <v>280</v>
       </c>
@@ -4823,11 +4193,7 @@
         </is>
       </c>
       <c r="M69" s="23"/>
-      <c r="N69" s="23" t="inlineStr">
-        <is>
-          <t>non_github</t>
-        </is>
-      </c>
+      <c r="N69" s="23"/>
       <c r="O69" s="23"/>
       <c r="P69" s="23"/>
       <c r="Q69" s="23"/>
@@ -4845,9 +4211,7 @@
       <c r="A70" s="24" t="s">
         <v>282</v>
       </c>
-      <c r="B70" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="B70" s="8"/>
       <c r="C70" s="25" t="s">
         <v>283</v>
       </c>
@@ -4875,11 +4239,7 @@
         </is>
       </c>
       <c r="M70" s="26"/>
-      <c r="N70" s="26" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+      <c r="N70" s="26"/>
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
       <c r="Q70" s="26"/>
@@ -4897,9 +4257,7 @@
       <c r="A71" s="24" t="s">
         <v>285</v>
       </c>
-      <c r="B71" s="15" t="s">
-        <v>50</v>
-      </c>
+      <c r="B71" s="15"/>
       <c r="C71" s="30" t="s">
         <v>286</v>
       </c>
@@ -4932,16 +4290,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M71" s="26" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="N71" s="26" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="M71" s="26"/>
+      <c r="N71" s="26"/>
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
       <c r="Q71" s="26"/>
@@ -4959,9 +4309,7 @@
       <c r="A72" s="11" t="s">
         <v>289</v>
       </c>
-      <c r="B72" s="15" t="s">
-        <v>50</v>
-      </c>
+      <c r="B72" s="15"/>
       <c r="C72" s="19" t="s">
         <v>290</v>
       </c>
@@ -4973,11 +4321,7 @@
         </is>
       </c>
       <c r="M72"/>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
+      <c r="N72"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="C73" s="7"/>
@@ -7426,9 +6770,7 @@
       <c r="A4" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="46" t="s">
-        <v>50</v>
-      </c>
+      <c r="B4" s="46"/>
       <c r="C4" s="7" t="s">
         <v>167</v>
       </c>
@@ -7455,16 +6797,8 @@
           <t>Stale</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>2025-09-04T19:12:30Z</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="K4"/>
+      <c r="L4"/>
       <c r="AA4" s="42"/>
       <c r="AB4" s="42"/>
       <c r="AC4" s="42"/>
@@ -7473,9 +6807,7 @@
       <c r="A5" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="B5" s="46" t="s">
-        <v>50</v>
-      </c>
+      <c r="B5" s="46"/>
       <c r="C5" s="7" t="s">
         <v>191</v>
       </c>
@@ -7502,16 +6834,8 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>2021-08-25T21:55:35Z</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="K5"/>
+      <c r="L5"/>
       <c r="AA5" s="42"/>
       <c r="AB5" s="42"/>
       <c r="AC5" s="42"/>
@@ -7520,9 +6844,7 @@
       <c r="A6" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="B6" s="46" t="s">
-        <v>50</v>
-      </c>
+      <c r="B6" s="46"/>
       <c r="C6" s="7" t="s">
         <v>171</v>
       </c>
@@ -7550,11 +6872,7 @@
         </is>
       </c>
       <c r="K6"/>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>non_github</t>
-        </is>
-      </c>
+      <c r="L6"/>
       <c r="AA6" s="42"/>
       <c r="AB6" s="42"/>
       <c r="AC6" s="42"/>
@@ -7563,9 +6881,7 @@
       <c r="A7" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="46" t="s">
-        <v>50</v>
-      </c>
+      <c r="B7" s="46"/>
       <c r="C7" s="7" t="s">
         <v>85</v>
       </c>
@@ -7592,16 +6908,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>2026-06-03T17:01:17Z</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>readme</t>
-        </is>
-      </c>
+      <c r="K7"/>
+      <c r="L7"/>
       <c r="AA7" s="42"/>
       <c r="AB7" s="42"/>
       <c r="AC7" s="42"/>
@@ -7610,9 +6918,7 @@
       <c r="A8" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="B8" s="46" t="s">
-        <v>50</v>
-      </c>
+      <c r="B8" s="46"/>
       <c r="C8" s="7" t="s">
         <v>187</v>
       </c>
@@ -7639,16 +6945,8 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>2026-05-27T00:39:03Z</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>idea_file</t>
-        </is>
-      </c>
+      <c r="K8"/>
+      <c r="L8"/>
       <c r="AA8" s="42"/>
       <c r="AB8" s="42"/>
       <c r="AC8" s="42"/>

</xml_diff>

<commit_message>
chore: refresh project workbook
</commit_message>
<xml_diff>
--- a/sources/Public Invention Projects.xlsx
+++ b/sources/Public Invention Projects.xlsx
@@ -1852,7 +1852,11 @@
       <c r="A2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="8"/>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C2" s="7" t="s">
         <v>13</v>
       </c>
@@ -1879,14 +1883,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M2"/>
-      <c r="N2"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="8"/>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C3" s="7" t="s">
         <v>19</v>
       </c>
@@ -1913,14 +1929,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M3"/>
-      <c r="N3"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="8"/>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C4" s="7" t="s">
         <v>23</v>
       </c>
@@ -1947,14 +1975,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M4"/>
-      <c r="N4"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="8"/>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C5" s="7" t="s">
         <v>27</v>
       </c>
@@ -1981,14 +2021,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M5"/>
-      <c r="N5"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="8"/>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C6" s="7" t="s">
         <v>31</v>
       </c>
@@ -2015,14 +2067,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M6"/>
-      <c r="N6"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="8"/>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C7" s="7" t="s">
         <v>31</v>
       </c>
@@ -2049,14 +2113,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M7"/>
-      <c r="N7"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="8"/>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C8" s="7" t="s">
         <v>38</v>
       </c>
@@ -2083,14 +2159,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M8"/>
-      <c r="N8"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="8"/>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C9" s="7" t="s">
         <v>42</v>
       </c>
@@ -2117,14 +2205,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M9"/>
-      <c r="N9"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="8"/>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C10" s="7" t="s">
         <v>46</v>
       </c>
@@ -2151,14 +2251,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M10"/>
-      <c r="N10"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="28.5" customHeight="1">
       <c r="A11" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="8"/>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C11" s="7" t="s">
         <v>51</v>
       </c>
@@ -2191,14 +2303,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M11"/>
-      <c r="N11"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="8"/>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C12" s="7" t="s">
         <v>56</v>
       </c>
@@ -2231,14 +2355,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M12"/>
-      <c r="N12"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="8"/>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C13" s="7" t="s">
         <v>60</v>
       </c>
@@ -2265,14 +2401,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M13"/>
-      <c r="N13"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="8"/>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C14" s="7" t="s">
         <v>64</v>
       </c>
@@ -2299,14 +2447,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M14"/>
-      <c r="N14"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="29.25" customHeight="1">
       <c r="A15" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B15" s="8"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
       <c r="C15" s="7" t="s">
         <v>68</v>
       </c>
@@ -2333,14 +2493,26 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M15"/>
-      <c r="N15"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>June 2020</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B16" s="8"/>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C16" s="7" t="s">
         <v>73</v>
       </c>
@@ -2373,14 +2545,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M16"/>
-      <c r="N16"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="8"/>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C17" s="7" t="s">
         <v>77</v>
       </c>
@@ -2407,14 +2591,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M17"/>
-      <c r="N17"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B18" s="8"/>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C18" s="7" t="s">
         <v>81</v>
       </c>
@@ -2447,14 +2643,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M18"/>
-      <c r="N18"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="42.75" customHeight="1">
       <c r="A19" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B19" s="8"/>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C19" s="7" t="s">
         <v>85</v>
       </c>
@@ -2487,14 +2695,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M19"/>
-      <c r="N19"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="8"/>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C20" s="7" t="s">
         <v>89</v>
       </c>
@@ -2521,14 +2741,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M20"/>
-      <c r="N20"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B21" s="8"/>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C21" s="7" t="s">
         <v>94</v>
       </c>
@@ -2555,14 +2787,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M21"/>
-      <c r="N21"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B22" s="8"/>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C22" s="7" t="s">
         <v>98</v>
       </c>
@@ -2589,14 +2833,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M22"/>
-      <c r="N22"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B23" s="8"/>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C23" s="7" t="s">
         <v>102</v>
       </c>
@@ -2623,14 +2879,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M23"/>
-      <c r="N23"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B24" s="8"/>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C24" s="7" t="s">
         <v>107</v>
       </c>
@@ -2657,14 +2925,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M24"/>
-      <c r="N24"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="B25" s="8"/>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C25" s="7" t="s">
         <v>110</v>
       </c>
@@ -2691,14 +2971,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M25"/>
-      <c r="N25"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="B26" s="8"/>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C26" s="7" t="s">
         <v>115</v>
       </c>
@@ -2725,14 +3017,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M26"/>
-      <c r="N26"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B27" s="8"/>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C27" s="7" t="s">
         <v>120</v>
       </c>
@@ -2757,14 +3061,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M27"/>
-      <c r="N27"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="B28" s="8"/>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C28" s="7" t="s">
         <v>123</v>
       </c>
@@ -2791,14 +3107,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M28"/>
-      <c r="N28"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B29" s="8"/>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C29" s="7" t="s">
         <v>127</v>
       </c>
@@ -2825,14 +3153,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M29"/>
-      <c r="N29"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B30" s="15"/>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C30" s="7" t="s">
         <v>131</v>
       </c>
@@ -2865,14 +3205,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M30"/>
-      <c r="N30"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="41.25" customHeight="1">
       <c r="A31" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="B31" s="8"/>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C31" s="7" t="s">
         <v>136</v>
       </c>
@@ -2899,14 +3251,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M31"/>
-      <c r="N31"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="8"/>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C32" s="7" t="s">
         <v>140</v>
       </c>
@@ -2933,14 +3297,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M32"/>
-      <c r="N32"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="B33" s="15"/>
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
       <c r="C33" s="7" t="s">
         <v>146</v>
       </c>
@@ -2967,14 +3343,26 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M33"/>
-      <c r="N33"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>October 2024</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="33.0" customHeight="1">
       <c r="A34" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="B34" s="8"/>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C34" s="7" t="s">
         <v>150</v>
       </c>
@@ -3001,14 +3389,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M34"/>
-      <c r="N34"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="29.25" customHeight="1">
       <c r="A35" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="B35" s="8"/>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C35" s="7" t="s">
         <v>154</v>
       </c>
@@ -3036,13 +3436,21 @@
         </is>
       </c>
       <c r="M35"/>
-      <c r="N35"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>non_github</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="31.5" customHeight="1">
       <c r="A37" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="B37" s="8"/>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C37" s="7" t="s">
         <v>159</v>
       </c>
@@ -3069,14 +3477,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M37"/>
-      <c r="N37"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="27.75" customHeight="1">
       <c r="A38" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="B38" s="8"/>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
       <c r="C38" s="7" t="s">
         <v>163</v>
       </c>
@@ -3109,14 +3529,26 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M38"/>
-      <c r="N38"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>September 2023</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
       <c r="A39" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="B39" s="8"/>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Stale</t>
+        </is>
+      </c>
       <c r="C39" s="7" t="s">
         <v>167</v>
       </c>
@@ -3149,14 +3581,26 @@
           <t>Stale</t>
         </is>
       </c>
-      <c r="M39"/>
-      <c r="N39"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>September 2025</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="B40" s="15"/>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C40" s="7" t="s">
         <v>171</v>
       </c>
@@ -3184,13 +3628,21 @@
         </is>
       </c>
       <c r="M40"/>
-      <c r="N40"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>non_github</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="B41" s="8"/>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C41" s="7" t="s">
         <v>175</v>
       </c>
@@ -3216,13 +3668,21 @@
         </is>
       </c>
       <c r="M41"/>
-      <c r="N41"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="B42" s="8"/>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C42" s="7" t="s">
         <v>178</v>
       </c>
@@ -3248,13 +3708,21 @@
         </is>
       </c>
       <c r="M42"/>
-      <c r="N42"/>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="B43" s="8"/>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C43" s="7" t="s">
         <v>181</v>
       </c>
@@ -3280,13 +3748,21 @@
         </is>
       </c>
       <c r="M43"/>
-      <c r="N43"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="B44" s="8"/>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C44" s="7" t="s">
         <v>184</v>
       </c>
@@ -3308,14 +3784,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M44"/>
-      <c r="N44"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="B45" s="8"/>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C45" s="7" t="s">
         <v>187</v>
       </c>
@@ -3348,14 +3836,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M45"/>
-      <c r="N45"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="B46" s="15"/>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
       <c r="C46" s="7" t="s">
         <v>191</v>
       </c>
@@ -3388,14 +3888,26 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M46"/>
-      <c r="N46"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>August 2021</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="B47" s="8"/>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
       <c r="C47" s="7" t="s">
         <v>195</v>
       </c>
@@ -3422,14 +3934,26 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M47"/>
-      <c r="N47"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>June 2021</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="27.0" customHeight="1">
       <c r="A48" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="B48" s="8"/>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C48" s="7" t="s">
         <v>199</v>
       </c>
@@ -3456,14 +3980,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M48"/>
-      <c r="N48"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="B49" s="8"/>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C49" s="7" t="s">
         <v>203</v>
       </c>
@@ -3490,14 +4026,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M49"/>
-      <c r="N49"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="B50" s="8"/>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C50" s="7" t="s">
         <v>207</v>
       </c>
@@ -3524,14 +4072,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M50"/>
-      <c r="N50"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="B51" s="15"/>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
       <c r="C51" s="7" t="s">
         <v>211</v>
       </c>
@@ -3558,14 +4118,26 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M51"/>
-      <c r="N51"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>January 2023</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="B52" s="15"/>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C52" s="7" t="s">
         <v>216</v>
       </c>
@@ -3590,14 +4162,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M52"/>
-      <c r="N52"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="B53" s="15"/>
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
       <c r="C53" s="7" t="s">
         <v>218</v>
       </c>
@@ -3622,14 +4206,26 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M53"/>
-      <c r="N53"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>August 2021</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="B54" s="8"/>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C54" s="7" t="s">
         <v>221</v>
       </c>
@@ -3656,14 +4252,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M54"/>
-      <c r="N54"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="B55" s="15"/>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C55" s="7" t="s">
         <v>225</v>
       </c>
@@ -3697,13 +4305,21 @@
         </is>
       </c>
       <c r="M55"/>
-      <c r="N55"/>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>non_github</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="B56" s="15"/>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C56" s="7" t="s">
         <v>230</v>
       </c>
@@ -3736,14 +4352,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M56"/>
-      <c r="N56"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="B57" s="8"/>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C57" s="7" t="s">
         <v>234</v>
       </c>
@@ -3769,13 +4397,21 @@
         </is>
       </c>
       <c r="M57"/>
-      <c r="N57"/>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="B58" s="8"/>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C58" s="7" t="s">
         <v>237</v>
       </c>
@@ -3801,13 +4437,21 @@
         </is>
       </c>
       <c r="M58"/>
-      <c r="N58"/>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="B59" s="15"/>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C59" s="7" t="s">
         <v>240</v>
       </c>
@@ -3834,14 +4478,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M59"/>
-      <c r="N59"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="8" t="s">
         <v>243</v>
       </c>
-      <c r="B60" s="8"/>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C60" s="7" t="s">
         <v>244</v>
       </c>
@@ -3868,14 +4524,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M60"/>
-      <c r="N60"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="B61" s="15"/>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C61" s="7" t="s">
         <v>248</v>
       </c>
@@ -3902,14 +4570,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M61"/>
-      <c r="N61"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="B62" s="8"/>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C62" s="7" t="s">
         <v>252</v>
       </c>
@@ -3936,14 +4616,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M62"/>
-      <c r="N62"/>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="8" t="s">
         <v>255</v>
       </c>
-      <c r="B63" s="8"/>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C63" s="7" t="s">
         <v>256</v>
       </c>
@@ -3970,14 +4662,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M63"/>
-      <c r="N63"/>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="B64" s="15"/>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
       <c r="C64" s="7" t="s">
         <v>260</v>
       </c>
@@ -4004,14 +4708,26 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M64"/>
-      <c r="N64"/>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>June 2023</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="15" t="s">
         <v>263</v>
       </c>
-      <c r="B65" s="15"/>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C65" s="7" t="s">
         <v>264</v>
       </c>
@@ -4044,14 +4760,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M65"/>
-      <c r="N65"/>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="B66" s="8"/>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
       <c r="C66" s="7" t="s">
         <v>268</v>
       </c>
@@ -4078,14 +4806,26 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="M66"/>
-      <c r="N66"/>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>May 2024</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="B67" s="15"/>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C67" s="19" t="s">
         <v>272</v>
       </c>
@@ -4118,14 +4858,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M67"/>
-      <c r="N67"/>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>February 2026</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="21" t="s">
         <v>275</v>
       </c>
-      <c r="B68" s="8"/>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C68" s="19" t="s">
         <v>276</v>
       </c>
@@ -4152,14 +4904,26 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M68"/>
-      <c r="N68"/>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="21" t="s">
         <v>279</v>
       </c>
-      <c r="B69" s="15"/>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C69" s="19" t="s">
         <v>280</v>
       </c>
@@ -4193,7 +4957,11 @@
         </is>
       </c>
       <c r="M69" s="23"/>
-      <c r="N69" s="23"/>
+      <c r="N69" s="23" t="inlineStr">
+        <is>
+          <t>non_github</t>
+        </is>
+      </c>
       <c r="O69" s="23"/>
       <c r="P69" s="23"/>
       <c r="Q69" s="23"/>
@@ -4211,7 +4979,11 @@
       <c r="A70" s="24" t="s">
         <v>282</v>
       </c>
-      <c r="B70" s="8"/>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C70" s="25" t="s">
         <v>283</v>
       </c>
@@ -4239,7 +5011,11 @@
         </is>
       </c>
       <c r="M70" s="26"/>
-      <c r="N70" s="26"/>
+      <c r="N70" s="26" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
       <c r="O70" s="26"/>
       <c r="P70" s="26"/>
       <c r="Q70" s="26"/>
@@ -4257,7 +5033,11 @@
       <c r="A71" s="24" t="s">
         <v>285</v>
       </c>
-      <c r="B71" s="15"/>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C71" s="30" t="s">
         <v>286</v>
       </c>
@@ -4290,8 +5070,16 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="M71" s="26"/>
-      <c r="N71" s="26"/>
+      <c r="M71" s="26" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="N71" s="26" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
       <c r="O71" s="26"/>
       <c r="P71" s="26"/>
       <c r="Q71" s="26"/>
@@ -4309,7 +5097,11 @@
       <c r="A72" s="11" t="s">
         <v>289</v>
       </c>
-      <c r="B72" s="15"/>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C72" s="19" t="s">
         <v>290</v>
       </c>
@@ -4321,7 +5113,11 @@
         </is>
       </c>
       <c r="M72"/>
-      <c r="N72"/>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="C73" s="7"/>
@@ -6770,7 +7566,11 @@
       <c r="A4" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="46"/>
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>Stale</t>
+        </is>
+      </c>
       <c r="C4" s="7" t="s">
         <v>167</v>
       </c>
@@ -6797,8 +7597,16 @@
           <t>Stale</t>
         </is>
       </c>
-      <c r="K4"/>
-      <c r="L4"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>September 2025</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
       <c r="AA4" s="42"/>
       <c r="AB4" s="42"/>
       <c r="AC4" s="42"/>
@@ -6807,7 +7615,11 @@
       <c r="A5" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="B5" s="46"/>
+      <c r="B5" s="46" t="inlineStr">
+        <is>
+          <t>Dormant</t>
+        </is>
+      </c>
       <c r="C5" s="7" t="s">
         <v>191</v>
       </c>
@@ -6834,8 +7646,16 @@
           <t>Dormant</t>
         </is>
       </c>
-      <c r="K5"/>
-      <c r="L5"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>August 2021</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
       <c r="AA5" s="42"/>
       <c r="AB5" s="42"/>
       <c r="AC5" s="42"/>
@@ -6844,7 +7664,11 @@
       <c r="A6" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="B6" s="46"/>
+      <c r="B6" s="46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
       <c r="C6" s="7" t="s">
         <v>171</v>
       </c>
@@ -6872,7 +7696,11 @@
         </is>
       </c>
       <c r="K6"/>
-      <c r="L6"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>non_github</t>
+        </is>
+      </c>
       <c r="AA6" s="42"/>
       <c r="AB6" s="42"/>
       <c r="AC6" s="42"/>
@@ -6881,7 +7709,11 @@
       <c r="A7" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="46"/>
+      <c r="B7" s="46" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C7" s="7" t="s">
         <v>85</v>
       </c>
@@ -6908,8 +7740,16 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="K7"/>
-      <c r="L7"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>readme</t>
+        </is>
+      </c>
       <c r="AA7" s="42"/>
       <c r="AB7" s="42"/>
       <c r="AC7" s="42"/>
@@ -6918,7 +7758,11 @@
       <c r="A8" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="B8" s="46"/>
+      <c r="B8" s="46" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="C8" s="7" t="s">
         <v>187</v>
       </c>
@@ -6945,8 +7789,16 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="K8"/>
-      <c r="L8"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>idea_file</t>
+        </is>
+      </c>
       <c r="AA8" s="42"/>
       <c r="AB8" s="42"/>
       <c r="AC8" s="42"/>

</xml_diff>